<commit_message>
change from wide to long format, better for sklearn later on
</commit_message>
<xml_diff>
--- a/extracted_features/extracted_features.xlsx
+++ b/extracted_features/extracted_features.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29825"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9BAF9A27-B321-4D68-805D-7106CD653ED1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{3A898F8D-1C06-48A5-A7E7-3559CFEEF110}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="9">
   <si>
     <t>participant_id</t>
   </si>
@@ -42,22 +42,16 @@
     <t>age</t>
   </si>
   <si>
-    <t>perceived_topic_intimacy_c1</t>
+    <t>condition</t>
   </si>
   <si>
-    <t>perceived_topic_intimacy_c2</t>
+    <t>perceived_topic_intimacy</t>
   </si>
   <si>
-    <t>personal_discomfort_c1</t>
+    <t>personal_discomfort</t>
   </si>
   <si>
-    <t>personal_discomfort_c2</t>
-  </si>
-  <si>
-    <t>revealing_personal_information_c1</t>
-  </si>
-  <si>
-    <t>revealing_personal_information_c2</t>
+    <t>revealing_personal_information</t>
   </si>
   <si>
     <t>M</t>
@@ -415,16 +409,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I26"/>
+  <dimension ref="A1:G51"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="27.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="22.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="33" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="24.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="29.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:7">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -446,83 +443,65 @@
       <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9">
+    </row>
+    <row r="2" spans="1:7">
       <c r="A2">
         <v>4</v>
       </c>
       <c r="B2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C2">
         <v>23</v>
       </c>
       <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2">
         <v>5</v>
-      </c>
-      <c r="E2">
-        <v>4</v>
       </c>
       <c r="F2">
         <v>1.571</v>
       </c>
       <c r="G2">
-        <v>1</v>
-      </c>
-      <c r="H2">
         <v>1.25</v>
       </c>
-      <c r="I2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9">
+    </row>
+    <row r="3" spans="1:7">
       <c r="A3">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3">
+        <v>23</v>
+      </c>
+      <c r="D3">
+        <v>2</v>
+      </c>
+      <c r="E3">
+        <v>4</v>
+      </c>
+      <c r="F3">
+        <v>1</v>
+      </c>
+      <c r="G3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7">
+      <c r="A4">
         <v>5</v>
       </c>
-      <c r="B3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C3">
+      <c r="B4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4">
         <v>20</v>
       </c>
-      <c r="D3">
-        <v>3</v>
-      </c>
-      <c r="E3">
-        <v>4</v>
-      </c>
-      <c r="F3">
-        <v>1.143</v>
-      </c>
-      <c r="G3">
-        <v>2.4289999999999998</v>
-      </c>
-      <c r="H3">
-        <v>1.25</v>
-      </c>
-      <c r="I3">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9">
-      <c r="A4">
-        <v>6</v>
-      </c>
-      <c r="B4" t="s">
-        <v>10</v>
-      </c>
-      <c r="C4">
-        <v>27</v>
-      </c>
       <c r="D4">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E4">
         <v>3</v>
@@ -531,259 +510,205 @@
         <v>1.143</v>
       </c>
       <c r="G4">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7">
+      <c r="A5">
+        <v>5</v>
+      </c>
+      <c r="B5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5">
+        <v>20</v>
+      </c>
+      <c r="D5">
+        <v>2</v>
+      </c>
+      <c r="E5">
+        <v>4</v>
+      </c>
+      <c r="F5">
+        <v>2.4289999999999998</v>
+      </c>
+      <c r="G5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
+      <c r="A6">
+        <v>6</v>
+      </c>
+      <c r="B6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6">
+        <v>27</v>
+      </c>
+      <c r="D6">
+        <v>1</v>
+      </c>
+      <c r="E6">
+        <v>4</v>
+      </c>
+      <c r="F6">
+        <v>1.143</v>
+      </c>
+      <c r="G6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>8</v>
+      </c>
+      <c r="C7">
+        <v>27</v>
+      </c>
+      <c r="D7">
+        <v>2</v>
+      </c>
+      <c r="E7">
+        <v>3</v>
+      </c>
+      <c r="F7">
         <v>1.286</v>
       </c>
-      <c r="H4">
-        <v>1</v>
-      </c>
-      <c r="I4">
+      <c r="G7">
         <v>2.75</v>
       </c>
     </row>
-    <row r="5" spans="1:9">
-      <c r="A5">
-        <v>7</v>
-      </c>
-      <c r="B5" t="s">
-        <v>10</v>
-      </c>
-      <c r="C5">
+    <row r="8" spans="1:7">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C8">
         <v>21</v>
       </c>
-      <c r="D5">
-        <v>1</v>
-      </c>
-      <c r="E5">
+      <c r="D8">
+        <v>1</v>
+      </c>
+      <c r="E8">
+        <v>1</v>
+      </c>
+      <c r="F8">
+        <v>1</v>
+      </c>
+      <c r="G8">
+        <v>1.75</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7">
+      <c r="A9">
+        <v>7</v>
+      </c>
+      <c r="B9" t="s">
+        <v>8</v>
+      </c>
+      <c r="C9">
+        <v>21</v>
+      </c>
+      <c r="D9">
+        <v>2</v>
+      </c>
+      <c r="E9">
         <v>3</v>
       </c>
-      <c r="F5">
-        <v>1</v>
-      </c>
-      <c r="G5">
-        <v>1</v>
-      </c>
-      <c r="H5">
+      <c r="F9">
+        <v>1</v>
+      </c>
+      <c r="G9">
         <v>1.75</v>
       </c>
-      <c r="I5">
-        <v>1.75</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9">
-      <c r="A6">
+    </row>
+    <row r="10" spans="1:7">
+      <c r="A10">
         <v>9</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C10">
+        <v>26</v>
+      </c>
+      <c r="D10">
+        <v>1</v>
+      </c>
+      <c r="E10">
+        <v>4</v>
+      </c>
+      <c r="F10">
+        <v>1.714</v>
+      </c>
+      <c r="G10">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7">
+      <c r="A11">
         <v>9</v>
       </c>
-      <c r="C6">
+      <c r="B11" t="s">
+        <v>7</v>
+      </c>
+      <c r="C11">
         <v>26</v>
       </c>
-      <c r="D6">
-        <v>4</v>
-      </c>
-      <c r="E6">
-        <v>2</v>
-      </c>
-      <c r="F6">
-        <v>1.714</v>
-      </c>
-      <c r="G6">
+      <c r="D11">
+        <v>2</v>
+      </c>
+      <c r="E11">
+        <v>2</v>
+      </c>
+      <c r="F11">
         <v>1.286</v>
       </c>
-      <c r="H6">
-        <v>2</v>
-      </c>
-      <c r="I6">
+      <c r="G11">
         <v>1.5</v>
       </c>
     </row>
-    <row r="7" spans="1:9">
-      <c r="A7">
+    <row r="12" spans="1:7">
+      <c r="A12">
         <v>11</v>
       </c>
-      <c r="B7" t="s">
-        <v>10</v>
-      </c>
-      <c r="C7">
+      <c r="B12" t="s">
+        <v>8</v>
+      </c>
+      <c r="C12">
         <v>28</v>
       </c>
-      <c r="D7">
-        <v>2</v>
-      </c>
-      <c r="E7">
-        <v>4</v>
-      </c>
-      <c r="F7">
-        <v>1</v>
-      </c>
-      <c r="G7">
-        <v>1.286</v>
-      </c>
-      <c r="H7">
-        <v>1</v>
-      </c>
-      <c r="I7">
-        <v>2.25</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9">
-      <c r="A8">
-        <v>12</v>
-      </c>
-      <c r="B8" t="s">
-        <v>10</v>
-      </c>
-      <c r="C8">
-        <v>19</v>
-      </c>
-      <c r="D8">
-        <v>2</v>
-      </c>
-      <c r="E8">
-        <v>5</v>
-      </c>
-      <c r="F8">
-        <v>1.143</v>
-      </c>
-      <c r="G8">
-        <v>2.5710000000000002</v>
-      </c>
-      <c r="H8">
-        <v>3.25</v>
-      </c>
-      <c r="I8">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9">
-      <c r="A9">
-        <v>13</v>
-      </c>
-      <c r="B9" t="s">
-        <v>10</v>
-      </c>
-      <c r="C9">
-        <v>19</v>
-      </c>
-      <c r="D9">
-        <v>2</v>
-      </c>
-      <c r="E9">
-        <v>5</v>
-      </c>
-      <c r="F9">
-        <v>1.143</v>
-      </c>
-      <c r="G9">
-        <v>2.4289999999999998</v>
-      </c>
-      <c r="H9">
-        <v>1.5</v>
-      </c>
-      <c r="I9">
-        <v>3.25</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9">
-      <c r="A10">
-        <v>14</v>
-      </c>
-      <c r="B10" t="s">
-        <v>10</v>
-      </c>
-      <c r="C10">
-        <v>24</v>
-      </c>
-      <c r="D10">
-        <v>4</v>
-      </c>
-      <c r="E10">
-        <v>3</v>
-      </c>
-      <c r="F10">
-        <v>1</v>
-      </c>
-      <c r="G10">
-        <v>1</v>
-      </c>
-      <c r="H10">
-        <v>3</v>
-      </c>
-      <c r="I10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9">
-      <c r="A11">
-        <v>15</v>
-      </c>
-      <c r="B11" t="s">
-        <v>9</v>
-      </c>
-      <c r="C11">
-        <v>29</v>
-      </c>
-      <c r="D11">
-        <v>3</v>
-      </c>
-      <c r="E11">
-        <v>4</v>
-      </c>
-      <c r="F11">
-        <v>1.143</v>
-      </c>
-      <c r="G11">
-        <v>2.1429999999999998</v>
-      </c>
-      <c r="H11">
-        <v>1.5</v>
-      </c>
-      <c r="I11">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9">
-      <c r="A12">
-        <v>16</v>
-      </c>
-      <c r="B12" t="s">
-        <v>10</v>
-      </c>
-      <c r="C12">
-        <v>24</v>
-      </c>
       <c r="D12">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E12">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F12">
-        <v>1.286</v>
+        <v>1</v>
       </c>
       <c r="G12">
-        <v>2.286</v>
-      </c>
-      <c r="H12">
-        <v>1.75</v>
-      </c>
-      <c r="I12">
-        <v>3.25</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7">
       <c r="A13">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="B13" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C13">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="D13">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E13">
         <v>4</v>
@@ -792,85 +717,67 @@
         <v>1.286</v>
       </c>
       <c r="G13">
+        <v>2.25</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7">
+      <c r="A14">
+        <v>12</v>
+      </c>
+      <c r="B14" t="s">
+        <v>8</v>
+      </c>
+      <c r="C14">
+        <v>19</v>
+      </c>
+      <c r="D14">
+        <v>1</v>
+      </c>
+      <c r="E14">
+        <v>2</v>
+      </c>
+      <c r="F14">
+        <v>1.143</v>
+      </c>
+      <c r="G14">
+        <v>3.25</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7">
+      <c r="A15">
+        <v>12</v>
+      </c>
+      <c r="B15" t="s">
+        <v>8</v>
+      </c>
+      <c r="C15">
+        <v>19</v>
+      </c>
+      <c r="D15">
+        <v>2</v>
+      </c>
+      <c r="E15">
+        <v>5</v>
+      </c>
+      <c r="F15">
         <v>2.5710000000000002</v>
       </c>
-      <c r="H13">
-        <v>1</v>
-      </c>
-      <c r="I13">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9">
-      <c r="A14">
-        <v>18</v>
-      </c>
-      <c r="B14" t="s">
-        <v>9</v>
-      </c>
-      <c r="C14">
-        <v>32</v>
-      </c>
-      <c r="D14">
-        <v>2</v>
-      </c>
-      <c r="E14">
-        <v>4</v>
-      </c>
-      <c r="F14">
-        <v>1.714</v>
-      </c>
-      <c r="G14">
-        <v>2.5710000000000002</v>
-      </c>
-      <c r="H14">
-        <v>1.75</v>
-      </c>
-      <c r="I14">
-        <v>2.25</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9">
-      <c r="A15">
+      <c r="G15">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7">
+      <c r="A16">
+        <v>13</v>
+      </c>
+      <c r="B16" t="s">
+        <v>8</v>
+      </c>
+      <c r="C16">
         <v>19</v>
       </c>
-      <c r="B15" t="s">
-        <v>9</v>
-      </c>
-      <c r="C15">
-        <v>35</v>
-      </c>
-      <c r="D15">
-        <v>1</v>
-      </c>
-      <c r="E15">
-        <v>4</v>
-      </c>
-      <c r="F15">
-        <v>1</v>
-      </c>
-      <c r="G15">
-        <v>1.286</v>
-      </c>
-      <c r="H15">
-        <v>1.25</v>
-      </c>
-      <c r="I15">
-        <v>1.25</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9">
-      <c r="A16">
-        <v>20</v>
-      </c>
-      <c r="B16" t="s">
-        <v>9</v>
-      </c>
-      <c r="C16">
-        <v>18</v>
-      </c>
       <c r="D16">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E16">
         <v>2</v>
@@ -879,85 +786,67 @@
         <v>1.143</v>
       </c>
       <c r="G16">
-        <v>2.1429999999999998</v>
-      </c>
-      <c r="H16">
-        <v>2.25</v>
-      </c>
-      <c r="I16">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7">
       <c r="A17">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="B17" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C17">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D17">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E17">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F17">
-        <v>1</v>
+        <v>2.4289999999999998</v>
       </c>
       <c r="G17">
-        <v>2.4289999999999998</v>
-      </c>
-      <c r="H17">
-        <v>2.5</v>
-      </c>
-      <c r="I17">
-        <v>3.75</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9">
+        <v>3.25</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7">
       <c r="A18">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="B18" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C18">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D18">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E18">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F18">
         <v>1</v>
       </c>
       <c r="G18">
-        <v>1.286</v>
-      </c>
-      <c r="H18">
-        <v>2.5</v>
-      </c>
-      <c r="I18">
-        <v>3.25</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7">
       <c r="A19">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="B19" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C19">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="D19">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E19">
         <v>3</v>
@@ -966,215 +855,742 @@
         <v>1</v>
       </c>
       <c r="G19">
-        <v>1.429</v>
-      </c>
-      <c r="H19">
-        <v>2.25</v>
-      </c>
-      <c r="I19">
         <v>3</v>
       </c>
     </row>
-    <row r="20" spans="1:9">
+    <row r="20" spans="1:7">
       <c r="A20">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="B20" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="C20">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D20">
+        <v>1</v>
+      </c>
+      <c r="E20">
         <v>3</v>
       </c>
-      <c r="E20">
-        <v>4</v>
-      </c>
       <c r="F20">
-        <v>1.571</v>
+        <v>1.143</v>
       </c>
       <c r="G20">
-        <v>3.1429999999999998</v>
-      </c>
-      <c r="H20">
         <v>1.5</v>
       </c>
-      <c r="I20">
-        <v>3.25</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9">
+    </row>
+    <row r="21" spans="1:7">
       <c r="A21">
-        <v>26</v>
+        <v>15</v>
       </c>
       <c r="B21" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="C21">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="D21">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E21">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F21">
-        <v>1.571</v>
+        <v>2.1429999999999998</v>
       </c>
       <c r="G21">
-        <v>1.143</v>
-      </c>
-      <c r="H21">
-        <v>1.25</v>
-      </c>
-      <c r="I21">
-        <v>2.25</v>
-      </c>
-    </row>
-    <row r="22" spans="1:9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7">
       <c r="A22">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="B22" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C22">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D22">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E22">
         <v>3</v>
       </c>
       <c r="F22">
+        <v>1.286</v>
+      </c>
+      <c r="G22">
+        <v>1.75</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7">
+      <c r="A23">
+        <v>16</v>
+      </c>
+      <c r="B23" t="s">
+        <v>8</v>
+      </c>
+      <c r="C23">
+        <v>24</v>
+      </c>
+      <c r="D23">
+        <v>2</v>
+      </c>
+      <c r="E23">
+        <v>5</v>
+      </c>
+      <c r="F23">
+        <v>2.286</v>
+      </c>
+      <c r="G23">
+        <v>3.25</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7">
+      <c r="A24">
+        <v>17</v>
+      </c>
+      <c r="B24" t="s">
+        <v>7</v>
+      </c>
+      <c r="C24">
+        <v>19</v>
+      </c>
+      <c r="D24">
+        <v>1</v>
+      </c>
+      <c r="E24">
+        <v>3</v>
+      </c>
+      <c r="F24">
+        <v>1.286</v>
+      </c>
+      <c r="G24">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7">
+      <c r="A25">
+        <v>17</v>
+      </c>
+      <c r="B25" t="s">
+        <v>7</v>
+      </c>
+      <c r="C25">
+        <v>19</v>
+      </c>
+      <c r="D25">
+        <v>2</v>
+      </c>
+      <c r="E25">
+        <v>4</v>
+      </c>
+      <c r="F25">
+        <v>2.5710000000000002</v>
+      </c>
+      <c r="G25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7">
+      <c r="A26">
+        <v>18</v>
+      </c>
+      <c r="B26" t="s">
+        <v>7</v>
+      </c>
+      <c r="C26">
+        <v>32</v>
+      </c>
+      <c r="D26">
+        <v>1</v>
+      </c>
+      <c r="E26">
+        <v>2</v>
+      </c>
+      <c r="F26">
+        <v>1.714</v>
+      </c>
+      <c r="G26">
+        <v>1.75</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7">
+      <c r="A27">
+        <v>18</v>
+      </c>
+      <c r="B27" t="s">
+        <v>7</v>
+      </c>
+      <c r="C27">
+        <v>32</v>
+      </c>
+      <c r="D27">
+        <v>2</v>
+      </c>
+      <c r="E27">
+        <v>4</v>
+      </c>
+      <c r="F27">
+        <v>2.5710000000000002</v>
+      </c>
+      <c r="G27">
+        <v>2.25</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7">
+      <c r="A28">
+        <v>19</v>
+      </c>
+      <c r="B28" t="s">
+        <v>7</v>
+      </c>
+      <c r="C28">
+        <v>35</v>
+      </c>
+      <c r="D28">
+        <v>1</v>
+      </c>
+      <c r="E28">
+        <v>1</v>
+      </c>
+      <c r="F28">
+        <v>1</v>
+      </c>
+      <c r="G28">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7">
+      <c r="A29">
+        <v>19</v>
+      </c>
+      <c r="B29" t="s">
+        <v>7</v>
+      </c>
+      <c r="C29">
+        <v>35</v>
+      </c>
+      <c r="D29">
+        <v>2</v>
+      </c>
+      <c r="E29">
+        <v>4</v>
+      </c>
+      <c r="F29">
+        <v>1.286</v>
+      </c>
+      <c r="G29">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7">
+      <c r="A30">
+        <v>20</v>
+      </c>
+      <c r="B30" t="s">
+        <v>7</v>
+      </c>
+      <c r="C30">
+        <v>18</v>
+      </c>
+      <c r="D30">
+        <v>1</v>
+      </c>
+      <c r="E30">
+        <v>4</v>
+      </c>
+      <c r="F30">
+        <v>1.143</v>
+      </c>
+      <c r="G30">
+        <v>2.25</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7">
+      <c r="A31">
+        <v>20</v>
+      </c>
+      <c r="B31" t="s">
+        <v>7</v>
+      </c>
+      <c r="C31">
+        <v>18</v>
+      </c>
+      <c r="D31">
+        <v>2</v>
+      </c>
+      <c r="E31">
+        <v>2</v>
+      </c>
+      <c r="F31">
+        <v>2.1429999999999998</v>
+      </c>
+      <c r="G31">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7">
+      <c r="A32">
+        <v>21</v>
+      </c>
+      <c r="B32" t="s">
+        <v>7</v>
+      </c>
+      <c r="C32">
+        <v>18</v>
+      </c>
+      <c r="D32">
+        <v>1</v>
+      </c>
+      <c r="E32">
+        <v>1</v>
+      </c>
+      <c r="F32">
+        <v>1</v>
+      </c>
+      <c r="G32">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7">
+      <c r="A33">
+        <v>21</v>
+      </c>
+      <c r="B33" t="s">
+        <v>7</v>
+      </c>
+      <c r="C33">
+        <v>18</v>
+      </c>
+      <c r="D33">
+        <v>2</v>
+      </c>
+      <c r="E33">
+        <v>4</v>
+      </c>
+      <c r="F33">
+        <v>2.4289999999999998</v>
+      </c>
+      <c r="G33">
+        <v>3.75</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7">
+      <c r="A34">
+        <v>22</v>
+      </c>
+      <c r="B34" t="s">
+        <v>8</v>
+      </c>
+      <c r="C34">
+        <v>23</v>
+      </c>
+      <c r="D34">
+        <v>1</v>
+      </c>
+      <c r="E34">
+        <v>4</v>
+      </c>
+      <c r="F34">
+        <v>1</v>
+      </c>
+      <c r="G34">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7">
+      <c r="A35">
+        <v>22</v>
+      </c>
+      <c r="B35" t="s">
+        <v>8</v>
+      </c>
+      <c r="C35">
+        <v>23</v>
+      </c>
+      <c r="D35">
+        <v>2</v>
+      </c>
+      <c r="E35">
+        <v>5</v>
+      </c>
+      <c r="F35">
+        <v>1.286</v>
+      </c>
+      <c r="G35">
+        <v>3.25</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7">
+      <c r="A36">
+        <v>23</v>
+      </c>
+      <c r="B36" t="s">
+        <v>7</v>
+      </c>
+      <c r="C36">
+        <v>21</v>
+      </c>
+      <c r="D36">
+        <v>1</v>
+      </c>
+      <c r="E36">
+        <v>3</v>
+      </c>
+      <c r="F36">
+        <v>1</v>
+      </c>
+      <c r="G36">
+        <v>2.25</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7">
+      <c r="A37">
+        <v>23</v>
+      </c>
+      <c r="B37" t="s">
+        <v>7</v>
+      </c>
+      <c r="C37">
+        <v>21</v>
+      </c>
+      <c r="D37">
+        <v>2</v>
+      </c>
+      <c r="E37">
+        <v>3</v>
+      </c>
+      <c r="F37">
+        <v>1.429</v>
+      </c>
+      <c r="G37">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7">
+      <c r="A38">
+        <v>25</v>
+      </c>
+      <c r="B38" t="s">
+        <v>8</v>
+      </c>
+      <c r="C38">
+        <v>27</v>
+      </c>
+      <c r="D38">
+        <v>1</v>
+      </c>
+      <c r="E38">
+        <v>3</v>
+      </c>
+      <c r="F38">
         <v>1.571</v>
       </c>
-      <c r="G22">
+      <c r="G38">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7">
+      <c r="A39">
+        <v>25</v>
+      </c>
+      <c r="B39" t="s">
+        <v>8</v>
+      </c>
+      <c r="C39">
+        <v>27</v>
+      </c>
+      <c r="D39">
+        <v>2</v>
+      </c>
+      <c r="E39">
+        <v>4</v>
+      </c>
+      <c r="F39">
+        <v>3.1429999999999998</v>
+      </c>
+      <c r="G39">
+        <v>3.25</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7">
+      <c r="A40">
+        <v>26</v>
+      </c>
+      <c r="B40" t="s">
+        <v>8</v>
+      </c>
+      <c r="C40">
+        <v>25</v>
+      </c>
+      <c r="D40">
+        <v>1</v>
+      </c>
+      <c r="E40">
+        <v>4</v>
+      </c>
+      <c r="F40">
+        <v>1.571</v>
+      </c>
+      <c r="G40">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7">
+      <c r="A41">
+        <v>26</v>
+      </c>
+      <c r="B41" t="s">
+        <v>8</v>
+      </c>
+      <c r="C41">
+        <v>25</v>
+      </c>
+      <c r="D41">
+        <v>2</v>
+      </c>
+      <c r="E41">
+        <v>2</v>
+      </c>
+      <c r="F41">
+        <v>1.143</v>
+      </c>
+      <c r="G41">
+        <v>2.25</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7">
+      <c r="A42">
+        <v>28</v>
+      </c>
+      <c r="B42" t="s">
+        <v>7</v>
+      </c>
+      <c r="C42">
+        <v>26</v>
+      </c>
+      <c r="D42">
+        <v>1</v>
+      </c>
+      <c r="E42">
+        <v>4</v>
+      </c>
+      <c r="F42">
+        <v>1.571</v>
+      </c>
+      <c r="G42">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7">
+      <c r="A43">
+        <v>28</v>
+      </c>
+      <c r="B43" t="s">
+        <v>7</v>
+      </c>
+      <c r="C43">
+        <v>26</v>
+      </c>
+      <c r="D43">
+        <v>2</v>
+      </c>
+      <c r="E43">
+        <v>3</v>
+      </c>
+      <c r="F43">
         <v>2.4289999999999998</v>
       </c>
-      <c r="H22">
-        <v>2</v>
-      </c>
-      <c r="I22">
+      <c r="G43">
         <v>3.25</v>
       </c>
     </row>
-    <row r="23" spans="1:9">
-      <c r="A23">
+    <row r="44" spans="1:7">
+      <c r="A44">
         <v>29</v>
       </c>
-      <c r="B23" t="s">
-        <v>9</v>
-      </c>
-      <c r="C23">
+      <c r="B44" t="s">
+        <v>7</v>
+      </c>
+      <c r="C44">
         <v>26</v>
       </c>
-      <c r="D23">
-        <v>2</v>
-      </c>
-      <c r="E23">
-        <v>4</v>
-      </c>
-      <c r="F23">
+      <c r="D44">
+        <v>1</v>
+      </c>
+      <c r="E44">
+        <v>2</v>
+      </c>
+      <c r="F44">
         <v>1.286</v>
       </c>
-      <c r="G23">
-        <v>1</v>
-      </c>
-      <c r="H23">
-        <v>1</v>
-      </c>
-      <c r="I23">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="24" spans="1:9">
-      <c r="A24">
+      <c r="G44">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7">
+      <c r="A45">
+        <v>29</v>
+      </c>
+      <c r="B45" t="s">
+        <v>7</v>
+      </c>
+      <c r="C45">
+        <v>26</v>
+      </c>
+      <c r="D45">
+        <v>2</v>
+      </c>
+      <c r="E45">
+        <v>4</v>
+      </c>
+      <c r="F45">
+        <v>1</v>
+      </c>
+      <c r="G45">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7">
+      <c r="A46">
         <v>30</v>
       </c>
-      <c r="B24" t="s">
-        <v>10</v>
-      </c>
-      <c r="C24">
+      <c r="B46" t="s">
+        <v>8</v>
+      </c>
+      <c r="C46">
         <v>22</v>
       </c>
-      <c r="D24">
+      <c r="D46">
+        <v>1</v>
+      </c>
+      <c r="E46">
         <v>3</v>
       </c>
-      <c r="E24">
-        <v>2</v>
-      </c>
-      <c r="F24">
+      <c r="F46">
         <v>1.571</v>
       </c>
-      <c r="G24">
+      <c r="G46">
+        <v>1.75</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7">
+      <c r="A47">
+        <v>30</v>
+      </c>
+      <c r="B47" t="s">
+        <v>8</v>
+      </c>
+      <c r="C47">
+        <v>22</v>
+      </c>
+      <c r="D47">
+        <v>2</v>
+      </c>
+      <c r="E47">
+        <v>2</v>
+      </c>
+      <c r="F47">
         <v>1.286</v>
       </c>
-      <c r="H24">
+      <c r="G47">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7">
+      <c r="A48">
+        <v>31</v>
+      </c>
+      <c r="B48" t="s">
+        <v>8</v>
+      </c>
+      <c r="C48">
+        <v>25</v>
+      </c>
+      <c r="D48">
+        <v>1</v>
+      </c>
+      <c r="E48">
+        <v>1</v>
+      </c>
+      <c r="F48">
+        <v>1</v>
+      </c>
+      <c r="G48">
         <v>1.75</v>
       </c>
-      <c r="I24">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="25" spans="1:9">
-      <c r="A25">
+    </row>
+    <row r="49" spans="1:7">
+      <c r="A49">
         <v>31</v>
       </c>
-      <c r="B25" t="s">
-        <v>10</v>
-      </c>
-      <c r="C25">
+      <c r="B49" t="s">
+        <v>8</v>
+      </c>
+      <c r="C49">
         <v>25</v>
       </c>
-      <c r="D25">
-        <v>1</v>
-      </c>
-      <c r="E25">
-        <v>4</v>
-      </c>
-      <c r="F25">
-        <v>1</v>
-      </c>
-      <c r="G25">
+      <c r="D49">
+        <v>2</v>
+      </c>
+      <c r="E49">
+        <v>4</v>
+      </c>
+      <c r="F49">
         <v>2.4289999999999998</v>
       </c>
-      <c r="H25">
-        <v>1.75</v>
-      </c>
-      <c r="I25">
+      <c r="G49">
         <v>3.5</v>
       </c>
     </row>
-    <row r="26" spans="1:9">
-      <c r="A26">
+    <row r="50" spans="1:7">
+      <c r="A50">
         <v>32</v>
       </c>
-      <c r="B26" t="s">
-        <v>10</v>
-      </c>
-      <c r="C26">
+      <c r="B50" t="s">
+        <v>8</v>
+      </c>
+      <c r="C50">
         <v>36</v>
       </c>
-      <c r="D26">
+      <c r="D50">
+        <v>1</v>
+      </c>
+      <c r="E50">
         <v>3</v>
       </c>
-      <c r="E26">
+      <c r="F50">
+        <v>1.429</v>
+      </c>
+      <c r="G50">
+        <v>2.75</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7">
+      <c r="A51">
+        <v>32</v>
+      </c>
+      <c r="B51" t="s">
+        <v>8</v>
+      </c>
+      <c r="C51">
+        <v>36</v>
+      </c>
+      <c r="D51">
+        <v>2</v>
+      </c>
+      <c r="E51">
         <v>5</v>
       </c>
-      <c r="F26">
-        <v>1.429</v>
-      </c>
-      <c r="G26">
+      <c r="F51">
         <v>3.714</v>
       </c>
-      <c r="H26">
-        <v>2.75</v>
-      </c>
-      <c r="I26">
+      <c r="G51">
         <v>4.5</v>
       </c>
     </row>
@@ -1184,6 +1600,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="db64c49b-6cfd-410c-b1e1-7c62a310e344" xsi:nil="true"/>
@@ -1192,15 +1617,6 @@
     </lcf76f155ced4ddcb4097134ff3c332f>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1445,11 +1861,11 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D9BE47D5-9894-4515-BA28-6EA0781EDD1D}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A0A45BD8-5424-4CD5-A579-D2B0627045AE}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A0A45BD8-5424-4CD5-A579-D2B0627045AE}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D9BE47D5-9894-4515-BA28-6EA0781EDD1D}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>